<commit_message>
changes for 3547 - added the manual review in check
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0918\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913C9FAB-7E65-4BD4-AAE6-0E543C6054C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D64A1AE3-9C17-42F6-AFA6-C0CA098F4359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3504,160 +3504,160 @@
     <t>Unable to validate Tenant Rights and Resource Guide (TRRG). Manual review is needed. </t>
   </si>
   <si>
-    <t>Unable to validate Housing History Disclosure. manual review required.</t>
-  </si>
-  <si>
-    <t>Live-In Attendant documented on the Income Calculation Worksheet. manual review required.</t>
-  </si>
-  <si>
-    <t>Applicant is a Dominium employee. manual review required.</t>
-  </si>
-  <si>
-    <t>Income type included that cannot be validated with automation. manual review required.</t>
-  </si>
-  <si>
-    <t>This application is a Section 811 unit. manual review required. </t>
-  </si>
-  <si>
-    <t>Unable to validate Income Calculation Worksheet. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Application Summary. manual review required.</t>
-  </si>
-  <si>
-    <t>Applicant reported a minor will live in the household less than 50% of the time. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Member Information Document. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Income &amp; Asset Questionnaire. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Self Certification of Non Employment. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Asset Self Certification &amp; Worksheet. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Affidavit of Student Financial Assistance. manual review required.</t>
-  </si>
-  <si>
-    <t>The applicant has indicated household contains all students by selecting 2 or 3 in Part A on the Student Certification. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Student Certification. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Annual Student Certification since there is Home unit . manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Certification of Zero Income. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate VAWA Acknowledgement. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Screening Document. manual review required.</t>
-  </si>
-  <si>
-    <t>Regular pay rate has increased across paystubs. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate paystubs. manual review required.</t>
-  </si>
-  <si>
-    <t>Verification of Employment - manual review required to ensure document was received via 3rd party.</t>
-  </si>
-  <si>
-    <t>Presently Employed has been listed as No on the Verification of Employment. manual review required.</t>
-  </si>
-  <si>
-    <t>Commission, bonuses, tips, other amount has been populated. manual review required.</t>
-  </si>
-  <si>
-    <t>Anticipated wage increase indicated on employment verification. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Verification of Employment. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Offer Letter. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Work Number. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Verification Services. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Self-Employment Certification. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Child Support Payment History. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Child Support Calcs. manual review required.</t>
-  </si>
-  <si>
-    <t>Overpayment listed on SS/SSI benefit letter. Documentation of months left on repayment is required. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Supplemental Security Income Letter. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Verification of Reccurring Cash Contribution. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Housing Demographic Reporting Form. manual review required.</t>
-  </si>
-  <si>
-    <t>Question 3 – Does any other member of your household receive a salary or other payments from this business has been documented as yes. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Certification of Self-Employment Income. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Profit/Loss Statement. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Applicant/Tenant Release and Consent. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Household Asset Breakdown. manual review required.</t>
-  </si>
-  <si>
-    <t>Presently Employed has been listed as No on the Verification of Employment. manual review required. </t>
-  </si>
-  <si>
-    <t>Unable to validate Employment Verification. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate the Certification of Student Status. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Regular Contributions Verification. manual review required.</t>
-  </si>
-  <si>
-    <t>Bank statements are included in the file. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Bank Statements. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Leave and Earnings Statement. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Veterans Affairs Benefits Letter. manual review required.</t>
-  </si>
-  <si>
-    <t>Unable to validate Release and Consent Form. manual review required. </t>
-  </si>
-  <si>
-    <t>Unable to validate Verification Services. manual review required. </t>
-  </si>
-  <si>
-    <t>Unable to validate Asset Certification of Net Family Assets. manual review required. </t>
+    <t>Unable to validate Housing History Disclosure. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Live-In Attendant documented on the Income Calculation Worksheet. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Applicant is a Dominium employee. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Income type included that cannot be validated with automation. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>This application is a Section 811 unit. Manual review is needed. </t>
+  </si>
+  <si>
+    <t>Unable to validate Income Calculation Worksheet. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Application Summary. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Applicant reported a minor will live in the household less than 50% of the time. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Member Information Document. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Income &amp; Asset Questionnaire. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Self Certification of Non Employment. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Asset Self Certification &amp; Worksheet. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Affidavit of Student Financial Assistance. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>The applicant has indicated household contains all students by selecting 2 or 3 in Part A on the Student Certification. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Student Certification. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Annual Student Certification since there is Home unit . Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Certification of Zero Income. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate VAWA Acknowledgement. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Screening Document. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Regular pay rate has increased across paystubs. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate paystubs. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Verification of Employment - manual review is needed to ensure document was received via 3rd party.</t>
+  </si>
+  <si>
+    <t>Presently Employed has been listed as No on the Verification of Employment. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Commission, bonuses, tips, other amount has been populated. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Anticipated wage increase indicated on employment verification. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Verification of Employment. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Offer Letter. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Work Number. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Verification Services. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Self-Employment Certification. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Child Support Payment History. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Child Support Calcs. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Overpayment listed on SS/SSI benefit letter. Documentation of months left on repayment is required. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Supplemental Security Income Letter. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Verification of Reccurring Cash Contribution. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Housing Demographic Reporting Form. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Question 3 – Does any other member of your household receive a salary or other payments from this business has been documented as yes. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Certification of Self-Employment Income. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Profit/Loss Statement. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Applicant/Tenant Release and Consent. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Household Asset Breakdown. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Presently Employed has been listed as No on the Verification of Employment. Manual review is needed. </t>
+  </si>
+  <si>
+    <t>Unable to validate Employment Verification. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate the Certification of Student Status. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Regular Contributions Verification. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Bank statements are included in the file. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Bank Statements. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Leave and Earnings Statement. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Veterans Affairs Benefits Letter. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>Unable to validate Release and Consent Form. Manual review is needed. </t>
+  </si>
+  <si>
+    <t>Unable to validate Verification Services. Manual review is needed. </t>
+  </si>
+  <si>
+    <t>Unable to validate Asset Certification of Net Family Assets. Manual review is needed. </t>
   </si>
 </sst>
 </file>
@@ -8567,7 +8567,7 @@
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
     <col min="2" max="2" width="153.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="97" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75">

</xml_diff>

<commit_message>
changes in Yardi library and also updated the config file
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B0A448-0804-48DE-ADD4-44ED023E2214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5753B921-D182-4E7D-86D4-3E8A41725FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1506" uniqueCount="1207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1510" uniqueCount="1209">
   <si>
     <t>Name</t>
   </si>
@@ -3664,6 +3664,12 @@
   </si>
   <si>
     <t>Unable to validate Verification of Recurring Cash Contribution. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>DelayAfterTime</t>
+  </si>
+  <si>
+    <t>ElementTimeout</t>
   </si>
 </sst>
 </file>
@@ -7138,7 +7144,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1014"/>
+  <dimension ref="A1:Z1016"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -7553,70 +7559,84 @@
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>910</v>
+        <v>1207</v>
       </c>
       <c r="B48" t="s">
-        <v>910</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>1047</v>
+        <v>1208</v>
       </c>
       <c r="B49" t="s">
-        <v>1047</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>1048</v>
+        <v>910</v>
       </c>
       <c r="B50" t="s">
-        <v>1048</v>
+        <v>910</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1">
       <c r="A51" t="s">
-        <v>1119</v>
+        <v>1047</v>
       </c>
       <c r="B51" t="s">
-        <v>1119</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>1122</v>
+        <v>1048</v>
       </c>
       <c r="B52" t="s">
-        <v>1122</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>1123</v>
+        <v>1119</v>
       </c>
       <c r="B53" t="s">
-        <v>1123</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="B54" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1">
       <c r="A55" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A56" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1124</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A57" t="s">
         <v>1197</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B57" t="s">
         <v>1197</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
@@ -8574,6 +8594,8 @@
     <row r="1012" ht="14.25" customHeight="1"/>
     <row r="1013" ht="14.25" customHeight="1"/>
     <row r="1014" ht="14.25" customHeight="1"/>
+    <row r="1015" ht="14.25" customHeight="1"/>
+    <row r="1016" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
changes in yardi library and in the code to save the documents
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5753B921-D182-4E7D-86D4-3E8A41725FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA54ECE3-234E-4A49-89C5-C04F508E26B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="16740" windowHeight="8250" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1510" uniqueCount="1209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="1211">
   <si>
     <t>Name</t>
   </si>
@@ -3670,6 +3670,12 @@
   </si>
   <si>
     <t>ElementTimeout</t>
+  </si>
+  <si>
+    <t>UnsupportedIncomeTypesFilePath</t>
+  </si>
+  <si>
+    <t>TX_VSAVerificationProperties</t>
   </si>
 </sst>
 </file>
@@ -7637,8 +7643,22 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A58" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1209</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A59" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1210</v>
+      </c>
+    </row>
     <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="62" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
changes to library and also added an activity from library for filtering the datatable
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F4B661-C6EA-4597-A366-9AD29E0AD47D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E141BA89-9856-4851-B091-C0A47A82B201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22560" windowHeight="11655" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1704" uniqueCount="1400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1706" uniqueCount="1401">
   <si>
     <t>Name</t>
   </si>
@@ -4243,6 +4243,9 @@
   </si>
   <si>
     <t>The applicant has indicated all household contains all students on the Income Calculation Worksheet. Manual review is needed.</t>
+  </si>
+  <si>
+    <t>COLACalcDate</t>
   </si>
 </sst>
 </file>
@@ -8233,7 +8236,14 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A60" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B60" t="s">
+        <v>1400</v>
+      </c>
+    </row>
     <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="63" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>